<commit_message>
add missing files:Ap Voucher advance initial testing done and changes for bringing Ar and Ap common parts in one place.
</commit_message>
<xml_diff>
--- a/src/test/resources/MasterTestData.xlsx
+++ b/src/test/resources/MasterTestData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>testcasename</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>TC101</t>
+  </si>
+  <si>
+    <t>createApVoucherAdvancePayment</t>
   </si>
 </sst>
 </file>
@@ -991,8 +994,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="5"/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="22.4285714285714" customWidth="1"/>
     <col min="2" max="2" width="14.4380952380952" customWidth="1"/>
@@ -1049,6 +1052,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4">
+        <v>200</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>

</xml_diff>

<commit_message>
General Voucher create test cases for mandatory and regression.testing is done majority of test cases passed
</commit_message>
<xml_diff>
--- a/src/test/resources/MasterTestData.xlsx
+++ b/src/test/resources/MasterTestData.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>testcasename</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>FIN-AP-ADV-TDS-CEPT</t>
+  </si>
+  <si>
+    <t>createGeneralVoucher</t>
+  </si>
+  <si>
+    <t>GV_TC01</t>
   </si>
 </sst>
 </file>
@@ -1013,8 +1019,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="5"/>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="7" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="35.2857142857143" customWidth="1"/>
     <col min="2" max="2" width="14.4380952380952" customWidth="1"/>
@@ -1115,6 +1121,17 @@
         <v>1</v>
       </c>
     </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait" useFirstPageNumber="1"/>

</xml_diff>